<commit_message>
restored missing files after reset
</commit_message>
<xml_diff>
--- a/Iwaniuk_etal_2001/Iwaniuk_etal_2001_table2_snapshot.xlsx
+++ b/Iwaniuk_etal_2001/Iwaniuk_etal_2001_table2_snapshot.xlsx
@@ -1577,8 +1577,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009B0162F312A93D41AE706303C1572F17" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="66af2654134d243f62aac8e2b322f1d6">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8e1efd23-f4ba-42d2-85fd-6a510437bae6" xmlns:ns3="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2bc3adf68671d86faa9c37249f400344" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009B0162F312A93D41AE706303C1572F17" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d42a73f51a03135be35f4acb272f8cf1">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8e1efd23-f4ba-42d2-85fd-6a510437bae6" xmlns:ns3="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2ea21b36c10eaa86a5cb337ec7f4e0a6" ns2:_="" ns3:_="">
     <xsd:import namespace="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
     <xsd:import namespace="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
     <xsd:element name="properties">
@@ -1602,6 +1602,8 @@
                 <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -1676,6 +1678,16 @@
     <xsd:element name="MediaServiceSearchProperties" ma:index="23" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="24" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="25" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
@@ -1828,23 +1840,19 @@
 </FormTemplates>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="8e1efd23-f4ba-42d2-85fd-6a510437bae6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4520FAFC-1D95-44A4-A356-BEF761B55D4E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
-    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E543E138-354F-4876-8346-8CEF808ECB64}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1853,4 +1861,8 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C8A34ACF-C079-4F2B-B680-7B64E26AC36E}"/>
 </file>
</xml_diff>